<commit_message>
list only the data files that carry every sheet the models need
list_data_files offered any .xlsx in data/, so input_asis.xlsx showed up in
the interface even though it is the raw monthly extraction and has none of
the weekly contract sheets. Check the sheet names before listing a file.

Lower MIN_LOT_SHIFT_CAP to 0.25 so the minimum lot stays near a two hour run,
and document in the README which sheets of input_asis_ajustado.xlsx are real
and which are synthesised, with the four dimensions the operation does not
record still open in TODO.md.
</commit_message>
<xml_diff>
--- a/data/input_asis_ajustado.xlsx
+++ b/data/input_asis_ajustado.xlsx
@@ -2771,7 +2771,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>63.3489270386268</v>
+        <v>31.6744635193134</v>
       </c>
     </row>
     <row r="3">
@@ -2786,7 +2786,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>33.48159392789372</v>
+        <v>16.74079696394686</v>
       </c>
     </row>
     <row r="4">
@@ -2801,7 +2801,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>12.8</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="5">
@@ -2816,7 +2816,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>30.00661384774368</v>
+        <v>15.00330692387184</v>
       </c>
     </row>
     <row r="6">
@@ -2831,7 +2831,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>61.3427125506072</v>
+        <v>30.6713562753036</v>
       </c>
     </row>
     <row r="7">
@@ -2846,7 +2846,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>103.5525904897088</v>
+        <v>51.7762952448544</v>
       </c>
     </row>
     <row r="8">
@@ -2861,7 +2861,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>68.47521517140839</v>
+        <v>34.2376075857042</v>
       </c>
     </row>
     <row r="9">
@@ -2876,7 +2876,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>51.4685446009388</v>
+        <v>25.7342723004694</v>
       </c>
     </row>
     <row r="10">
@@ -2891,7 +2891,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>31.65959664908472</v>
+        <v>15.82979832454236</v>
       </c>
     </row>
     <row r="11">
@@ -2906,7 +2906,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>60.0523061755448</v>
+        <v>30.0261530877724</v>
       </c>
     </row>
     <row r="12">
@@ -2936,7 +2936,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>16.36241771025962</v>
+        <v>8.930597958191539</v>
       </c>
     </row>
     <row r="14">
@@ -2951,7 +2951,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>113.0301468068368</v>
+        <v>56.5150734034184</v>
       </c>
     </row>
     <row r="15">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>45.6368970910228</v>
+        <v>22.8184485455114</v>
       </c>
     </row>
     <row r="17">
@@ -2996,7 +2996,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>83.1505917159764</v>
+        <v>41.5752958579882</v>
       </c>
     </row>
     <row r="18">
@@ -3011,7 +3011,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>82.4798929570608</v>
+        <v>41.2399464785304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>